<commit_message>
style: agregar bordes negros definidos y fila automatica de Total General
</commit_message>
<xml_diff>
--- a/Reporte_Parametrizado_Final.xlsx
+++ b/Reporte_Parametrizado_Final.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,6 +31,11 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -48,7 +53,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -56,16 +61,33 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -431,11 +453,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -451,23 +473,34 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Ana</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B2" s="3" t="n">
         <v>3900</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Carlos</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B3" s="3" t="n">
         <v>6100</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Total General</t>
+        </is>
+      </c>
+      <c r="B4" s="5">
+        <f>SUM(B2:B3)</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>